<commit_message>
Add the population pyramid
</commit_message>
<xml_diff>
--- a/402/402 _4.xlsx
+++ b/402/402 _4.xlsx
@@ -1,22 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Lecture notes 2025\B.Stat 402\Practical\402 practical problem (Demography) By Anika\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8495E5CA-A417-4009-8366-E5D142DBE74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{20D72148-5E42-49FC-A07B-9894CD21D95A}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19005" windowHeight="6615" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="popuPyramid-25" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="51">
   <si>
     <t>Age Group</t>
   </si>
@@ -223,11 +218,14 @@
   <si>
     <t xml:space="preserve">Total </t>
   </si>
+  <si>
+    <t>Sum</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -307,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -330,6 +328,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -339,10 +341,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,7 +360,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -408,26 +407,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -535,7 +514,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-9294-4395-847D-9B5BBBD4D7B8}"/>
             </c:ext>
@@ -640,7 +619,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-9294-4395-847D-9B5BBBD4D7B8}"/>
             </c:ext>
@@ -656,11 +635,11 @@
         </c:dLbls>
         <c:gapWidth val="0"/>
         <c:overlap val="100"/>
-        <c:axId val="1177615408"/>
-        <c:axId val="1177607248"/>
+        <c:axId val="181523968"/>
+        <c:axId val="181525504"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1177615408"/>
+        <c:axId val="181523968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -669,7 +648,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1177607248"/>
+        <c:crossAx val="181525504"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -677,7 +656,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1177607248"/>
+        <c:axId val="181525504"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -714,7 +693,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1177615408"/>
+        <c:crossAx val="181523968"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -760,7 +739,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -802,7 +781,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -816,6 +795,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -984,7 +964,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-4F28-40AC-BF85-64A98E05B041}"/>
             </c:ext>
@@ -1122,7 +1102,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-4F28-40AC-BF85-64A98E05B041}"/>
             </c:ext>
@@ -1138,11 +1118,11 @@
         </c:dLbls>
         <c:gapWidth val="40"/>
         <c:overlap val="100"/>
-        <c:axId val="1352589471"/>
-        <c:axId val="1352589951"/>
+        <c:axId val="182285824"/>
+        <c:axId val="182287360"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1352589471"/>
+        <c:axId val="182285824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1185,7 +1165,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1352589951"/>
+        <c:crossAx val="182287360"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1193,7 +1173,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1352589951"/>
+        <c:axId val="182287360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1244,12 +1224,13 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1352589471"/>
+        <c:crossAx val="182285824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:dispUnits>
           <c:builtInUnit val="hundreds"/>
           <c:dispUnitsLbl>
+            <c:layout/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1290,6 +1271,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1322,7 +1304,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -1355,6 +1337,373 @@
       <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Population Pyramid</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>2011</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$F$3:$F$19</c:f>
+              <c:strCache>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>0-4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5-9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10-14</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15-19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20-24</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25-29</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30-34</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35-39</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40-44</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45-49</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>50-54</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>55-59</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>60-64</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>65-69</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>70-74</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>75-79</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>80+</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$G$3:$G$19</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>-9.3093625589163953E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-8.6134245488796349E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-7.8841196479507006E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-7.3979163806647444E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-7.0737808691407736E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-6.8306792354977955E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-6.6781448771335739E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-6.5399106148659986E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6.206241705944264E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-5.8964062905169388E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-5.4674034076175659E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-5.2815021583611711E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-4.4687800302018028E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-4.0413024908860722E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-3.5204929910462333E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-2.6931847648682866E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-2.0973474275080461E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>2021</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$F$3:$F$19</c:f>
+              <c:strCache>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>0-4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5-9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10-14</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15-19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20-24</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25-29</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30-34</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35-39</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40-44</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45-49</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>50-54</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>55-59</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>60-64</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>65-69</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>70-74</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>75-79</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>80+</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$H$3:$H$19</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>9.3471484186961662E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.6461122872939541E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.949282372680154E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.7113974454243367E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.0290556108595165E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.7766826035547206E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.571045338343405E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.3467137762946962E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6.1130350658272929E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.8419677616851039E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.4026517860063843E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.2998331534007265E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.5099991120209001E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.0052530974113071E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5192013796391065E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.8041445256088499E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.1264762652533777E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="44"/>
+        <c:overlap val="100"/>
+        <c:axId val="33940992"/>
+        <c:axId val="34619392"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="33940992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:crossAx val="34619392"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="34619392"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="#,##0%;#,##0%" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="33940992"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
@@ -2470,7 +2819,7 @@
         <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96EC2522-890C-F826-9BB6-11D617C7ADAC}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96EC2522-890C-F826-9BB6-11D617C7ADAC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2495,26 +2844,61 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>536574</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>6350</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>260349</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>228599</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>561974</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4FCA1D0-5F80-FB6B-C1C6-9BCB78F2E9AE}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4FCA1D0-5F80-FB6B-C1C6-9BCB78F2E9AE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2821,41 +3205,41 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00C43188-C7B7-408A-918C-7B75C823A074}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="8.7265625" style="5"/>
-    <col min="5" max="5" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" style="5" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="5"/>
+    <col min="1" max="1" width="11.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="8.7109375" style="5"/>
+    <col min="5" max="5" width="12.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="8.7109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10"/>
+      <c r="C1" s="14"/>
       <c r="D1" s="1"/>
       <c r="E1" t="s">
         <v>18</v>
       </c>
       <c r="F1"/>
     </row>
-    <row r="2" spans="1:9" ht="15" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
+    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="14"/>
       <c r="B2" s="1">
         <v>2001</v>
       </c>
@@ -2870,7 +3254,7 @@
         <v>2011</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2895,7 +3279,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -2917,7 +3301,7 @@
         <v>12.616634268258817</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
@@ -2939,7 +3323,7 @@
         <v>11.555817828381006</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2961,7 +3345,7 @@
         <v>8.9287697861705073</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -2983,7 +3367,7 @@
         <v>9.2328519855595665</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -3005,7 +3389,7 @@
         <v>9.3578172729797284</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
@@ -3027,7 +3411,7 @@
         <v>7.2889475145792835</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -3049,7 +3433,7 @@
         <v>6.6342682588169959</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
@@ -3071,7 +3455,7 @@
         <v>5.7352124409886143</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
@@ -3093,7 +3477,7 @@
         <v>4.4293251874479314</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
@@ -3115,7 +3499,7 @@
         <v>3.85448486531519</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
@@ -3137,7 +3521,7 @@
         <v>2.4298805887253541</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
@@ -3159,7 +3543,7 @@
         <v>2.731185781727298</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
@@ -3181,7 +3565,7 @@
         <v>1.4669536239933352</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -3203,7 +3587,7 @@
         <v>1.5488753124132186</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
@@ -3225,7 +3609,7 @@
         <v>1.7328519855595668</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
@@ -3246,12 +3630,12 @@
         <v>99.999999999999986</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B22" s="5">
         <v>2001</v>
       </c>
@@ -3263,7 +3647,7 @@
         <v>125637</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B23" s="5">
         <v>2011</v>
       </c>
@@ -3275,7 +3659,7 @@
         <v>144040</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="5" t="s">
         <v>24</v>
       </c>
@@ -3284,17 +3668,17 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G25" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="8" t="s">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
       <c r="D26" s="5">
         <f>(D23-D22)/(D24*D22)</f>
         <v>1.4647755040314557E-2</v>
@@ -3306,68 +3690,68 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="8" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
       <c r="D27" s="5">
         <f>((D23/D22)^(1/D24))-1</f>
         <v>1.376327794788601E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="8" t="s">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
       <c r="D28" s="5">
         <f>(1/D24)*LN(D23/D22)</f>
         <v>1.3669424214124731E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B33" s="8" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
       <c r="F33" s="5">
         <f>LN(2)/LN(D27+1)</f>
         <v>50.707854969026918</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B34" s="8" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
       <c r="F34" s="5">
         <f>LN(2)/D28</f>
         <v>50.707854969027188</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B39" s="9" t="s">
+    <row r="39" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B39" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
       <c r="E39" s="7" t="s">
         <v>32</v>
       </c>
@@ -3376,10 +3760,10 @@
         <v>205226.01644420039</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
+    <row r="40" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
       <c r="E40" s="7" t="s">
         <v>33</v>
       </c>
@@ -3388,12 +3772,12 @@
         <v>226324.64280426945</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B41" s="9" t="s">
+    <row r="41" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B41" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
       <c r="E41" s="7" t="s">
         <v>32</v>
       </c>
@@ -3402,10 +3786,10 @@
         <v>214113.09162923857</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
+    <row r="42" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
       <c r="E42" s="7" t="s">
         <v>33</v>
       </c>
@@ -3414,12 +3798,12 @@
         <v>245475.85280033396</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B43" s="9" t="s">
+    <row r="43" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B43" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
       <c r="E43" s="7" t="s">
         <v>32</v>
       </c>
@@ -3428,10 +3812,10 @@
         <v>214113.0916292379</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
+    <row r="44" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
       <c r="E44" s="7" t="s">
         <v>33</v>
       </c>
@@ -3459,14 +3843,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4653A8F-45A2-4CA1-98CD-7A1A8B831C54}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="11"/>
+    <col min="1" max="1" width="8.7109375" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>40</v>
       </c>
@@ -3474,25 +3858,25 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:6" s="11" customFormat="1" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="11">
         <v>2011</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="11">
         <v>2021</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="11">
         <v>2001</v>
       </c>
-      <c r="F2" s="14">
+      <c r="F2" s="11">
         <v>2011</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B3">
@@ -3513,8 +3897,8 @@
         <v>9.3471484186961664</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B4">
@@ -3527,7 +3911,7 @@
         <v>16</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E19" si="0">-(B4/$B$20)*100</f>
+        <f t="shared" ref="E4:E18" si="0">-(B4/$B$20)*100</f>
         <v>-8.6134245488796353</v>
       </c>
       <c r="F4">
@@ -3535,8 +3919,8 @@
         <v>8.6461122872939544</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
       <c r="B5">
@@ -3557,8 +3941,8 @@
         <v>7.9492823726801536</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B6">
@@ -3579,8 +3963,8 @@
         <v>7.7113974454243364</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
         <v>4</v>
       </c>
       <c r="B7">
@@ -3601,8 +3985,8 @@
         <v>7.0290556108595164</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
@@ -3623,8 +4007,8 @@
         <v>6.776682603554721</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
       <c r="B9">
@@ -3645,8 +4029,8 @@
         <v>6.5710453383434047</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B10">
@@ -3667,8 +4051,8 @@
         <v>6.3467137762946964</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
+    <row r="11" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B11">
@@ -3689,8 +4073,8 @@
         <v>6.1130350658272929</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B12">
@@ -3711,8 +4095,8 @@
         <v>5.8419677616851038</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
+    <row r="13" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B13">
@@ -3733,8 +4117,8 @@
         <v>5.4026517860063841</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
+    <row r="14" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B14">
@@ -3755,8 +4139,8 @@
         <v>5.2998331534007264</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
+    <row r="15" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B15">
@@ -3777,8 +4161,8 @@
         <v>4.5099991120208998</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="11" t="s">
+    <row r="16" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B16">
@@ -3799,8 +4183,8 @@
         <v>4.0052530974113072</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
+    <row r="17" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B17">
@@ -3821,8 +4205,8 @@
         <v>3.5192013796391066</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
+    <row r="18" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A18" s="8" t="s">
         <v>41</v>
       </c>
       <c r="B18">
@@ -3843,8 +4227,8 @@
         <v>2.8041445256088497</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
+    <row r="19" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A19" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B19">
@@ -3865,8 +4249,8 @@
         <v>2.1264762652533777</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="11" t="s">
+    <row r="20" spans="1:6" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
         <v>49</v>
       </c>
       <c r="B20">
@@ -3886,29 +4270,467 @@
         <v>100.00000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="11" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="11" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="11" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
         <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="8"/>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="11">
+        <v>2011</v>
+      </c>
+      <c r="C2" s="11">
+        <v>2021</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11">
+        <v>2011</v>
+      </c>
+      <c r="H2" s="11">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>195300</v>
+      </c>
+      <c r="C3">
+        <v>200000</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="15">
+        <f>-B3/B$20</f>
+        <v>-9.3093625589163953E-2</v>
+      </c>
+      <c r="H3" s="15">
+        <f>C3/C$20</f>
+        <v>9.3471484186961662E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>180700</v>
+      </c>
+      <c r="C4">
+        <v>185000</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="15">
+        <f t="shared" ref="G4:G19" si="0">-B4/B$20</f>
+        <v>-8.6134245488796349E-2</v>
+      </c>
+      <c r="H4" s="15">
+        <f>C4/C$20</f>
+        <v>8.6461122872939541E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>165400</v>
+      </c>
+      <c r="C5">
+        <v>170090</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="15">
+        <f t="shared" si="0"/>
+        <v>-7.8841196479507006E-2</v>
+      </c>
+      <c r="H5" s="15">
+        <f t="shared" ref="H4:H19" si="1">C5/C$20</f>
+        <v>7.949282372680154E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>155200</v>
+      </c>
+      <c r="C6">
+        <v>165000</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="15">
+        <f t="shared" si="0"/>
+        <v>-7.3979163806647444E-2</v>
+      </c>
+      <c r="H6" s="15">
+        <f t="shared" si="1"/>
+        <v>7.7113974454243367E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>148400</v>
+      </c>
+      <c r="C7">
+        <v>150400</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="15">
+        <f t="shared" si="0"/>
+        <v>-7.0737808691407736E-2</v>
+      </c>
+      <c r="H7" s="15">
+        <f t="shared" si="1"/>
+        <v>7.0290556108595165E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>143300</v>
+      </c>
+      <c r="C8">
+        <v>145000</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="15">
+        <f t="shared" si="0"/>
+        <v>-6.8306792354977955E-2</v>
+      </c>
+      <c r="H8" s="15">
+        <f t="shared" si="1"/>
+        <v>6.7766826035547206E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>140100</v>
+      </c>
+      <c r="C9">
+        <v>140600</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="15">
+        <f t="shared" si="0"/>
+        <v>-6.6781448771335739E-2</v>
+      </c>
+      <c r="H9" s="15">
+        <f t="shared" si="1"/>
+        <v>6.571045338343405E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>137200</v>
+      </c>
+      <c r="C10">
+        <v>135800</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="15">
+        <f t="shared" si="0"/>
+        <v>-6.5399106148659986E-2</v>
+      </c>
+      <c r="H10" s="15">
+        <f t="shared" si="1"/>
+        <v>6.3467137762946962E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <v>130200</v>
+      </c>
+      <c r="C11">
+        <v>130800</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="15">
+        <f t="shared" si="0"/>
+        <v>-6.206241705944264E-2</v>
+      </c>
+      <c r="H11" s="15">
+        <f t="shared" si="1"/>
+        <v>6.1130350658272929E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>123700</v>
+      </c>
+      <c r="C12">
+        <v>125000</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="15">
+        <f t="shared" si="0"/>
+        <v>-5.8964062905169388E-2</v>
+      </c>
+      <c r="H12" s="15">
+        <f t="shared" si="1"/>
+        <v>5.8419677616851039E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>114700</v>
+      </c>
+      <c r="C13">
+        <v>115600</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="15">
+        <f t="shared" si="0"/>
+        <v>-5.4674034076175659E-2</v>
+      </c>
+      <c r="H13" s="15">
+        <f t="shared" si="1"/>
+        <v>5.4026517860063843E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14">
+        <v>110800</v>
+      </c>
+      <c r="C14">
+        <v>113400</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="15">
+        <f t="shared" si="0"/>
+        <v>-5.2815021583611711E-2</v>
+      </c>
+      <c r="H14" s="15">
+        <f t="shared" si="1"/>
+        <v>5.2998331534007265E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15">
+        <v>93750</v>
+      </c>
+      <c r="C15">
+        <v>96500</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="15">
+        <f t="shared" si="0"/>
+        <v>-4.4687800302018028E-2</v>
+      </c>
+      <c r="H15" s="15">
+        <f t="shared" si="1"/>
+        <v>4.5099991120209001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16">
+        <v>84782</v>
+      </c>
+      <c r="C16">
+        <v>85700</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="15">
+        <f t="shared" si="0"/>
+        <v>-4.0413024908860722E-2</v>
+      </c>
+      <c r="H16" s="15">
+        <f t="shared" si="1"/>
+        <v>4.0052530974113071E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17">
+        <v>73856</v>
+      </c>
+      <c r="C17">
+        <v>75300</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="15">
+        <f t="shared" si="0"/>
+        <v>-3.5204929910462333E-2</v>
+      </c>
+      <c r="H17" s="15">
+        <f t="shared" si="1"/>
+        <v>3.5192013796391065E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18">
+        <v>56500</v>
+      </c>
+      <c r="C18">
+        <v>60000</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="15">
+        <f t="shared" si="0"/>
+        <v>-2.6931847648682866E-2</v>
+      </c>
+      <c r="H18" s="15">
+        <f t="shared" si="1"/>
+        <v>2.8041445256088499E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19">
+        <v>44000</v>
+      </c>
+      <c r="C19">
+        <v>45500</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G19" s="15">
+        <f t="shared" si="0"/>
+        <v>-2.0973474275080461E-2</v>
+      </c>
+      <c r="H19" s="15">
+        <f t="shared" si="1"/>
+        <v>2.1264762652533777E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20">
+        <f>SUM(B3:B19)</f>
+        <v>2097888</v>
+      </c>
+      <c r="C20">
+        <f>SUM(C3:C19)</f>
+        <v>2139690</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G20" s="8">
+        <f>SUM(G3:G19)</f>
+        <v>-0.99999999999999978</v>
+      </c>
+      <c r="H20" s="8">
+        <f>SUM(H3:H19)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>